<commit_message>
Restore legacy labels in reviewed Jakarta Banten workbooks
</commit_message>
<xml_diff>
--- a/samples/ss_lbk_ingest.xlsx
+++ b/samples/ss_lbk_ingest.xlsx
@@ -835,7 +835,7 @@
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>Kembangan 150 kV</t>
+          <t>Kembangan (bus 150 kV)</t>
         </is>
       </c>
       <c r="C2" s="9" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>MTLAN</t>
+          <t>Metland</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>NSYAN</t>
+          <t>New Senayan</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>CLDUG</t>
+          <t>Ciledug</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>SNYAN</t>
+          <t>Senayan</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>ALTRA</t>
+          <t>Alam Sutera</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>DNYSA</t>
+          <t>Danayasa</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>CKUPA</t>
+          <t>Cikupa</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>SGS</t>
+          <t>Summarecon Gading Serpong</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>CURUG</t>
+          <t>Curug</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>JTAKE</t>
+          <t>Jatake</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>MAXIM</t>
+          <t>Maxim</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>New Balaraja 150 kV</t>
+          <t>New Balaraja (bus 150 kV)</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>TGBRU</t>
+          <t>Tangerang Baru</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>SVRNA</t>
+          <t>Suvarna Sutra</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>TLKGA</t>
+          <t>Teluknaga</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -2347,7 +2347,7 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>CNKNG</t>
+          <t>Cengkareng</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
@@ -2410,7 +2410,7 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>PSKMS</t>
+          <t>Pasar Kemis</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
@@ -2473,7 +2473,7 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>PSKBR</t>
+          <t>Pasar Kemis Baru</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>SPTAN (label suffix perlu cek)</t>
+          <t>Sepatan</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>TGRNG</t>
+          <t>Tangerang</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
@@ -2662,7 +2662,7 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>GJTGL</t>
+          <t>Gajah Tunggal</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
@@ -4986,7 +4986,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GITET New Cikupa (boundary)</t>
+          <t>GITET New Cikupa (rencana)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -5072,7 +5072,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tangerang Baru 3 (boundary)</t>
+          <t>Tangerang Baru 3 (belum energize)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -5115,7 +5115,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Jatake Baru (boundary)</t>
+          <t>Jatake Baru</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">

</xml_diff>

<commit_message>
Restore LBK voltage sources and add combined Muarakarang Durikosambi view
</commit_message>
<xml_diff>
--- a/samples/ss_lbk_ingest.xlsx
+++ b/samples/ss_lbk_ingest.xlsx
@@ -704,7 +704,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>KMBGN;NBRJA;ILKNG</t>
+          <t>GITET_KMBGN;GITET_NBRJA;ILKNG</t>
         </is>
       </c>
     </row>
@@ -719,7 +719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U32"/>
+  <dimension ref="A1:U38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -889,16 +889,8 @@
           <t>Root / source side</t>
         </is>
       </c>
-      <c r="P2" s="9" t="inlineStr">
-        <is>
-          <t>Rawan</t>
-        </is>
-      </c>
-      <c r="Q2" s="9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="P2" s="9" t="n"/>
+      <c r="Q2" s="9" t="n"/>
       <c r="R2" s="9" t="inlineStr">
         <is>
           <t>Jakarta &amp; Banten</t>
@@ -2817,6 +2809,376 @@
       </c>
       <c r="T32" s="9" t="n"/>
       <c r="U32" s="9" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>GITET Kembangan</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>GITET_KMBGN</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Busbar GITET</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>500 kV</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Historical LBK SLD: 500/150 kV source</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>SOURCE</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Rawan</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Banten</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>IBT 1 Kembangan</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>IBT 1 KMBGN</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>IBT 3-Winding</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>500/150 kV</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>GITET_KMBGN</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>KMBGN</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>1</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Historical LBK SLD: IBT unit</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>SOURCE_BOUNDARY</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Banten</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>IBT 2 Kembangan</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>IBT 2 KMBGN</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>IBT 3-Winding</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>500/150 kV</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>GITET_KMBGN</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>KMBGN</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>1</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Historical LBK SLD: IBT unit</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>SOURCE_BOUNDARY</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Banten</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>GITET New Balaraja</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>GITET_NBRJA</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Busbar GITET</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>500 kV</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Historical LBK SLD: 500/150 kV source</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>SOURCE</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Banten</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>IBT 1 New Balaraja</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>IBT 1 NBRJA</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>IBT 3-Winding</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>500/150 kV</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>GITET_NBRJA</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>NBRJA</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>1</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Historical LBK SLD: IBT unit</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>SOURCE_BOUNDARY</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Banten</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>IBT 2 New Balaraja</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>IBT 2 NBRJA</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>IBT 3-Winding</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>500/150 kV</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>GITET_NBRJA</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>NBRJA</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>1</v>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Historical LBK SLD: IBT unit</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>SOURCE_BOUNDARY</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Banten</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Restore LBK source pages and prevent boundary status leaking into neighbouring GI
</commit_message>
<xml_diff>
--- a/samples/ss_lbk_ingest.xlsx
+++ b/samples/ss_lbk_ingest.xlsx
@@ -660,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -694,17 +694,52 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FULL</t>
+          <t>KEMBANGAN</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SLD lengkap</t>
+          <t>Sisi Kembangan</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GITET_KMBGN;GITET_NBRJA;ILKNG</t>
+          <t>GITET_KMBGN</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Sisi Balaraja / Lontar</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GITET_NBRJA;LTKNG</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GABUNGAN</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Gabungan Lontar - Balaraja - Kembangan</t>
         </is>
       </c>
     </row>
@@ -719,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U38"/>
+  <dimension ref="A1:V42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -840,6 +875,11 @@
           <t>Longitude</t>
         </is>
       </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Sudut Pandang</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="n">
@@ -903,6 +943,11 @@
       </c>
       <c r="T2" s="9" t="n"/>
       <c r="U2" s="9" t="n"/>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="n">
@@ -966,6 +1011,11 @@
       </c>
       <c r="T3" s="9" t="n"/>
       <c r="U3" s="9" t="n"/>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="n">
@@ -1029,6 +1079,11 @@
       </c>
       <c r="T4" s="9" t="n"/>
       <c r="U4" s="9" t="n"/>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n">
@@ -1092,6 +1147,11 @@
       </c>
       <c r="T5" s="9" t="n"/>
       <c r="U5" s="9" t="n"/>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="n">
@@ -1163,6 +1223,11 @@
       </c>
       <c r="T6" s="9" t="n"/>
       <c r="U6" s="9" t="n"/>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="n">
@@ -1170,12 +1235,12 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>UUMI</t>
+          <t>Ulujami</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>UUMI</t>
+          <t>ULJMI</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
@@ -1226,6 +1291,11 @@
       </c>
       <c r="T7" s="9" t="n"/>
       <c r="U7" s="9" t="n"/>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="n">
@@ -1289,6 +1359,11 @@
       </c>
       <c r="T8" s="9" t="n"/>
       <c r="U8" s="9" t="n"/>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="n">
@@ -1352,6 +1427,11 @@
       </c>
       <c r="T9" s="9" t="n"/>
       <c r="U9" s="9" t="n"/>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="n">
@@ -1415,6 +1495,11 @@
       </c>
       <c r="T10" s="9" t="n"/>
       <c r="U10" s="9" t="n"/>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>KEMBANGAN;BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n">
@@ -1478,6 +1563,11 @@
       </c>
       <c r="T11" s="9" t="n"/>
       <c r="U11" s="9" t="n"/>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n">
@@ -1541,6 +1631,11 @@
       </c>
       <c r="T12" s="9" t="n"/>
       <c r="U12" s="9" t="n"/>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n">
@@ -1604,6 +1699,11 @@
       </c>
       <c r="T13" s="9" t="n"/>
       <c r="U13" s="9" t="n"/>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>KEMBANGAN;BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="n">
@@ -1667,6 +1767,11 @@
       </c>
       <c r="T14" s="9" t="n"/>
       <c r="U14" s="9" t="n"/>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n">
@@ -1730,6 +1835,11 @@
       </c>
       <c r="T15" s="9" t="n"/>
       <c r="U15" s="9" t="n"/>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="n">
@@ -1737,12 +1847,12 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Lontar / ILKNG</t>
+          <t>Lontar</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>ILKNG</t>
+          <t>LTKNG</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
@@ -1793,6 +1903,11 @@
       </c>
       <c r="T16" s="9" t="n"/>
       <c r="U16" s="9" t="n"/>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="n">
@@ -1800,12 +1915,12 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>DLRA</t>
+          <t>Balaraja</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>DLRA</t>
+          <t>BLRJA</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
@@ -1856,6 +1971,11 @@
       </c>
       <c r="T17" s="9" t="n"/>
       <c r="U17" s="9" t="n"/>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="n">
@@ -1863,12 +1983,12 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>SUJYA</t>
+          <t>Sindang Jaya</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>SUJYA</t>
+          <t>SDJYA</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
@@ -1919,6 +2039,11 @@
       </c>
       <c r="T18" s="9" t="n"/>
       <c r="U18" s="9" t="n"/>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="n">
@@ -1926,12 +2051,12 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>ILKNG2 / DADAP</t>
+          <t>Teluknaga 2 / Dadap</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>DADAP</t>
+          <t>TLKNG2</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
@@ -1982,6 +2107,11 @@
       </c>
       <c r="T19" s="9" t="n"/>
       <c r="U19" s="9" t="n"/>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="n">
@@ -2045,6 +2175,11 @@
       </c>
       <c r="T20" s="9" t="n"/>
       <c r="U20" s="9" t="n"/>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="n">
@@ -2108,6 +2243,11 @@
       </c>
       <c r="T21" s="9" t="n"/>
       <c r="U21" s="9" t="n"/>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>KEMBANGAN;BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="n">
@@ -2171,6 +2311,11 @@
       </c>
       <c r="T22" s="9" t="n"/>
       <c r="U22" s="9" t="n"/>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="n">
@@ -2178,12 +2323,12 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>CKDRU</t>
+          <t>Cikupa Baru</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>CKDRU</t>
+          <t>CKBRU</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
@@ -2234,6 +2379,11 @@
       </c>
       <c r="T23" s="9" t="n"/>
       <c r="U23" s="9" t="n"/>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="n">
@@ -2241,12 +2391,12 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>IIS</t>
+          <t>KTT ITS</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>IIS</t>
+          <t>ITS</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
@@ -2297,6 +2447,11 @@
       </c>
       <c r="T24" s="9" t="n"/>
       <c r="U24" s="9" t="n"/>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="n">
@@ -2304,12 +2459,12 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>SPTAR</t>
+          <t>Sepatan</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>SPTAR</t>
+          <t>SPTAN</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
@@ -2360,6 +2515,11 @@
       </c>
       <c r="T25" s="9" t="n"/>
       <c r="U25" s="9" t="n"/>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="n">
@@ -2431,6 +2591,11 @@
       </c>
       <c r="T26" s="9" t="n"/>
       <c r="U26" s="9" t="n"/>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="n">
@@ -2494,6 +2659,11 @@
       </c>
       <c r="T27" s="9" t="n"/>
       <c r="U27" s="9" t="n"/>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>KEMBANGAN;BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="n">
@@ -2557,6 +2727,11 @@
       </c>
       <c r="T28" s="9" t="n"/>
       <c r="U28" s="9" t="n"/>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="n">
@@ -2564,12 +2739,12 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Sepatan</t>
+          <t>Sepatan 2</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>SPTAN</t>
+          <t>SPTAN2</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
@@ -2620,6 +2795,11 @@
       </c>
       <c r="T29" s="9" t="n"/>
       <c r="U29" s="9" t="n"/>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="n">
@@ -2683,6 +2863,11 @@
       </c>
       <c r="T30" s="9" t="n"/>
       <c r="U30" s="9" t="n"/>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="n">
@@ -2746,6 +2931,11 @@
       </c>
       <c r="T31" s="9" t="n"/>
       <c r="U31" s="9" t="n"/>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="n">
@@ -2753,12 +2943,12 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>JTKDR</t>
+          <t>Jatake Baru</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>JTKDR</t>
+          <t>JTKBR</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
@@ -2809,6 +2999,11 @@
       </c>
       <c r="T32" s="9" t="n"/>
       <c r="U32" s="9" t="n"/>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>KEMBANGAN;BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2867,6 +3062,11 @@
           <t>Banten</t>
         </is>
       </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2933,6 +3133,11 @@
           <t>Banten</t>
         </is>
       </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2999,6 +3204,11 @@
           <t>Banten</t>
         </is>
       </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -3047,6 +3257,11 @@
           <t>Banten</t>
         </is>
       </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -3113,6 +3328,11 @@
           <t>Banten</t>
         </is>
       </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -3177,6 +3397,208 @@
       <c r="R38" t="inlineStr">
         <is>
           <t>Banten</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>PLTU Lontar</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>KIT_LTKNG</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Pembangkit</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Buku hal.70: generator above Lontar bus</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>SOURCE</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Banten</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>GIS PLTD Senayan</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>GIS PLTD SNY</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Busbar GIS</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Buku hal.69 and Tabel 2.3: PLTD tap on Senayan-Danayasa corridor</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Banten</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>PLTD Senayan</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>PLTD SNY</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Pembangkit</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Banten</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Tangerang Baru 3 (belum energize)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>TGBRU3</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Busbar GI</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Buku hal.70: black planned bus in Lontar-Sindang Jaya corridor; historical connection to Lontar</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Belum Operasi</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Banten</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q33"/>
+  <dimension ref="A1:R38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3290,6 +3712,11 @@
           <t>Catatan Sudut Pandang Sumber</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Sudut Pandang</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="n">
@@ -3298,7 +3725,7 @@
       <c r="B2" s="9" t="n"/>
       <c r="C2" s="9" t="inlineStr">
         <is>
-          <t>SUTT KMBGN - MTLAN</t>
+          <t>SKTT KMBGN - MTLAN</t>
         </is>
       </c>
       <c r="D2" s="9" t="inlineStr">
@@ -3353,6 +3780,11 @@
           <t>Kembangan | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="n">
@@ -3365,7 +3797,7 @@
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>SUTT KMBGN - NSYAN</t>
+          <t>SKTT KMBGN - NSYAN</t>
         </is>
       </c>
       <c r="D3" s="9" t="inlineStr">
@@ -3420,6 +3852,11 @@
           <t>Kembangan | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="n">
@@ -3428,7 +3865,7 @@
       <c r="B4" s="9" t="n"/>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>SUTT MTLAN - CLDUG</t>
+          <t>SKTT MTLAN - CLDUG</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
@@ -3483,6 +3920,11 @@
           <t>Kembangan | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n">
@@ -3491,7 +3933,7 @@
       <c r="B5" s="9" t="n"/>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>SUTT CLDUG - ALTRA</t>
+          <t>SKTT CLDUG - ALTRA</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
@@ -3546,6 +3988,11 @@
           <t>Kembangan | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="n">
@@ -3554,7 +4001,7 @@
       <c r="B6" s="9" t="n"/>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>SUTT ALTRA - SGS</t>
+          <t>SKTT ALTRA - SGS</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -3609,6 +4056,11 @@
           <t>Kembangan | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="n">
@@ -3617,7 +4069,7 @@
       <c r="B7" s="9" t="n"/>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>SUTT SGS - CURUG</t>
+          <t>SKTT SGS - CURUG</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
@@ -3672,6 +4124,11 @@
           <t>Kembangan | Same-tier tie | Accepted | Confidence High | U-shaped tie pada Tier-5</t>
         </is>
       </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="n">
@@ -3680,7 +4137,7 @@
       <c r="B8" s="9" t="n"/>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>SUTT CURUG - CKUPA</t>
+          <t>SKTT CURUG - CKUPA</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -3735,6 +4192,11 @@
           <t>Kembangan | Reverse-tier edge | Accepted | Confidence High | Naik dari Tier-5 ke Tier-4 pada layout sumber</t>
         </is>
       </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="n">
@@ -3747,7 +4209,7 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>SUTT NSYAN - SNYAN</t>
+          <t>SKTT NSYAN - SNYAN</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
@@ -3802,6 +4264,11 @@
           <t>Kembangan | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="n">
@@ -3810,7 +4277,7 @@
       <c r="B10" s="9" t="n"/>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>SUTT NSYAN - UUMI</t>
+          <t>SKTT NSYAN - ULJMI</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -3820,7 +4287,7 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>UUMI</t>
+          <t>ULJMI</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
@@ -3865,6 +4332,11 @@
           <t>Kembangan | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="n">
@@ -3873,7 +4345,7 @@
       <c r="B11" s="9" t="n"/>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>SUTT SNYAN - DNYSA</t>
+          <t>SKTT SNYAN - DNYSA</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
@@ -3893,7 +4365,7 @@
       </c>
       <c r="G11" s="9" t="n"/>
       <c r="H11" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
@@ -3928,6 +4400,11 @@
           <t>Kembangan | Core | Verify | Confidence Medium-High | Dua drop menuju DNYSA terlihat, tracing tetap perlu final check</t>
         </is>
       </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="n">
@@ -3995,6 +4472,11 @@
           <t>Kembangan + Balaraja boundary | Stitch | Accepted | Confidence High | JTAKE full bus di Kembangan, boundary di Balaraja</t>
         </is>
       </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n">
@@ -4058,6 +4540,11 @@
           <t>Kembangan | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="n">
@@ -4066,7 +4553,7 @@
       <c r="B14" s="9" t="n"/>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>SUTT NBRJA - DLRA</t>
+          <t>SUTT NBRJA - BLRJA</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
@@ -4076,7 +4563,7 @@
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>DLRA</t>
+          <t>BLRJA</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
@@ -4121,6 +4608,11 @@
           <t>Balaraja | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n">
@@ -4129,17 +4621,17 @@
       <c r="B15" s="9" t="n"/>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>SUTT ILKNG - SUJYA</t>
+          <t>SUTT LTKNG - SDJYA</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>ILKNG</t>
+          <t>LTKNG</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>SUJYA</t>
+          <t>SDJYA</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
@@ -4184,6 +4676,11 @@
           <t>Balaraja | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="n">
@@ -4192,17 +4689,17 @@
       <c r="B16" s="9" t="n"/>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>SUTT ILKNG - DADAP</t>
+          <t>SUTT LTKNG - TLKNG2</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>ILKNG</t>
+          <t>LTKNG</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>DADAP</t>
+          <t>TLKNG2</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
@@ -4247,6 +4744,11 @@
           <t>Balaraja | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="n">
@@ -4259,12 +4761,12 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>SUTT ILKNG - TGBRU</t>
+          <t>SUTT LTKNG - TGBRU</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>ILKNG</t>
+          <t>LTKNG</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -4314,6 +4816,11 @@
           <t>Balaraja | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="n">
@@ -4322,12 +4829,12 @@
       <c r="B18" s="9" t="n"/>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>SUTT DLRA - SVRNA</t>
+          <t>SUTT BLRJA - SVRNA</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>DLRA</t>
+          <t>BLRJA</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -4377,6 +4884,11 @@
           <t>Balaraja | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="n">
@@ -4385,12 +4897,12 @@
       <c r="B19" s="9" t="n"/>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>SUTT SUJYA - SVRNA</t>
+          <t>SUTT SDJYA - SVRNA</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>SUJYA</t>
+          <t>SDJYA</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
@@ -4440,6 +4952,11 @@
           <t>Balaraja | Core | Verify | Confidence Medium-High | Routing paralel kompleks di antara DLRA-SUJYA-SVRNA</t>
         </is>
       </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="n">
@@ -4448,12 +4965,12 @@
       <c r="B20" s="9" t="n"/>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>SUTT DADAP - TLKGA</t>
+          <t>SUTT TLKNG2 - TLKGA</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>DADAP</t>
+          <t>TLKNG2</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -4503,6 +5020,11 @@
           <t>Balaraja | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="n">
@@ -4511,7 +5033,7 @@
       <c r="B21" s="9" t="n"/>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>SUTT TGBRU - CKDRU</t>
+          <t>SUTT TGBRU - CKBRU</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
@@ -4521,7 +5043,7 @@
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>CKDRU</t>
+          <t>CKBRU</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
@@ -4566,6 +5088,11 @@
           <t>Balaraja | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="n">
@@ -4574,7 +5101,7 @@
       <c r="B22" s="9" t="n"/>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>SUTT TGBRU - IIS</t>
+          <t>SUTT TGBRU - ITS</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
@@ -4584,7 +5111,7 @@
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>IIS</t>
+          <t>ITS</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
@@ -4629,6 +5156,11 @@
           <t>Balaraja | Core | Accepted | Confidence High | Long routed pair</t>
         </is>
       </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="n">
@@ -4692,6 +5224,11 @@
           <t>Balaraja + Kembangan boundary | Stitch | Accepted | Confidence High | Menghubungkan dua PoV</t>
         </is>
       </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="n">
@@ -4755,6 +5292,11 @@
           <t>Balaraja + Kembangan boundary | Stitch | Accepted | Confidence High | PSKMS boundary di Kembangan, full bus di Balaraja</t>
         </is>
       </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="n">
@@ -4763,7 +5305,7 @@
       <c r="B25" s="9" t="n"/>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>SUTT TLKGA - SPTAR</t>
+          <t>SUTT TLKGA - SPTAN</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
@@ -4773,7 +5315,7 @@
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>SPTAR</t>
+          <t>SPTAN</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
@@ -4818,6 +5360,11 @@
           <t>Balaraja | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="n">
@@ -4826,12 +5373,12 @@
       <c r="B26" s="9" t="n"/>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>SUTT SPTAR - PSKBR</t>
+          <t>SUTT SPTAN - PSKBR</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>SPTAR</t>
+          <t>SPTAN</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -4881,6 +5428,11 @@
           <t>Balaraja | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="n">
@@ -4889,17 +5441,17 @@
       <c r="B27" s="9" t="n"/>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>SUTT SPTAR - SPTAN</t>
+          <t>SUTT SPTAN - SPTAN2</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>SPTAR</t>
+          <t>SPTAN</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>SPTAN</t>
+          <t>SPTAN2</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
@@ -4944,6 +5496,11 @@
           <t>Balaraja | Core | Verify | Confidence Medium | Kode bus Tier-5 perlu konfirmasi label</t>
         </is>
       </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="n">
@@ -4952,12 +5509,12 @@
       <c r="B28" s="9" t="n"/>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>SUTT CKDRU - CNKNG</t>
+          <t>SUTT CKBRU - CNKNG</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>CKDRU</t>
+          <t>CKBRU</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -5007,6 +5564,11 @@
           <t>Balaraja | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="n">
@@ -5070,6 +5632,11 @@
           <t>Balaraja | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="n">
@@ -5078,7 +5645,7 @@
       <c r="B30" s="9" t="n"/>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>SUTT TGRNG - JTKDR</t>
+          <t>SUTT TGRNG - JTKBR</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
@@ -5088,7 +5655,7 @@
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>JTKDR</t>
+          <t>JTKBR</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
@@ -5133,6 +5700,11 @@
           <t>Balaraja | Core | Accepted | Confidence High</t>
         </is>
       </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="n">
@@ -5188,12 +5760,17 @@
       </c>
       <c r="P31" s="9" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t>Ya</t>
         </is>
       </c>
       <c r="Q31" s="9" t="inlineStr">
         <is>
           <t>Balaraja | Same-tier tie | Verify | Confidence Medium | Kerawanan #3; jumlah sirkit final perlu konfirmasi</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
         </is>
       </c>
     </row>
@@ -5255,12 +5832,17 @@
       </c>
       <c r="P32" s="9" t="inlineStr">
         <is>
-          <t>Tidak</t>
+          <t>Ya</t>
         </is>
       </c>
       <c r="Q32" s="9" t="inlineStr">
         <is>
           <t>Balaraja | Core | Verify | Confidence Medium-High | Single line terlihat</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
         </is>
       </c>
     </row>
@@ -5322,12 +5904,312 @@
       </c>
       <c r="P33" s="9" t="inlineStr">
         <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="Q33" s="9" t="inlineStr">
+        <is>
+          <t>Balaraja | Core | Verify | Confidence Medium | Faint single route; perlu final check</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Outlet PLTU Lontar</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>KIT_LTKNG</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LTKNG</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>1</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Jakarta &amp; Banten</t>
+        </is>
+      </c>
+      <c r="N34" t="n">
+        <v>1</v>
+      </c>
+      <c r="O34" t="n">
+        <v>1</v>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
           <t>Tidak</t>
         </is>
       </c>
-      <c r="Q33" s="9" t="inlineStr">
-        <is>
-          <t>Balaraja | Core | Verify | Confidence Medium | Faint single route; perlu final check</t>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Outlet PLTD Senayan</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>PLTD SNY</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>GIS PLTD SNY</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>1</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Jakarta &amp; Banten</t>
+        </is>
+      </c>
+      <c r="N35" t="n">
+        <v>1</v>
+      </c>
+      <c r="O35" t="n">
+        <v>1</v>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>SKTT Senayan - GIS PLTD Senayan</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>SNYAN</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>GIS PLTD SNY</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="H36" t="n">
+        <v>1</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Jakarta &amp; Banten</t>
+        </is>
+      </c>
+      <c r="N36" t="n">
+        <v>3</v>
+      </c>
+      <c r="O36" t="n">
+        <v>3</v>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>SKTT GIS PLTD Senayan - Danayasa</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>GIS PLTD SNY</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>DNYSA</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="H37" t="n">
+        <v>1</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Jakarta &amp; Banten</t>
+        </is>
+      </c>
+      <c r="N37" t="n">
+        <v>3</v>
+      </c>
+      <c r="O37" t="n">
+        <v>4</v>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Ya</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>SUTT Lontar - Tangerang Baru 3</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>LTKNG</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>TGBRU3</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="H38" t="n">
+        <v>2</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Belum Operasi</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Jakarta &amp; Banten</t>
+        </is>
+      </c>
+      <c r="N38" t="n">
+        <v>1</v>
+      </c>
+      <c r="O38" t="n">
+        <v>2</v>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Tidak</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
         </is>
       </c>
     </row>
@@ -5342,7 +6224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5396,6 +6278,11 @@
           <t>Catatan Sudut Pandang Sumber</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Sudut Pandang</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -5439,6 +6326,11 @@
           <t>Boundary_External; source evidence</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -5446,17 +6338,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CKNN?</t>
+          <t>CKNDE</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CKNN? (label raster)</t>
+          <t>Cikande</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>DLRA</t>
+          <t>BLRJA</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -5474,12 +6366,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Belum Operasi</t>
+          <t>Beroperasi</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
           <t>Boundary_External; source evidence</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
         </is>
       </c>
     </row>
@@ -5489,17 +6386,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>TGBRU3</t>
+          <t>JTKBR</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tangerang Baru 3 (belum energize)</t>
+          <t>Jatake Baru</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SUJYA</t>
+          <t>JTAKE</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -5523,6 +6420,11 @@
       <c r="J4" t="inlineStr">
         <is>
           <t>Boundary_External; source evidence</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
         </is>
       </c>
     </row>
@@ -5532,22 +6434,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>JTKBR</t>
+          <t>BSH</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Jatake Baru</t>
+          <t>BSH (KTT / customer asset)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>JTAKE</t>
+          <t>CKBRU</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Boundary / external</t>
+          <t>KTT / customer</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -5560,12 +6462,17 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Belum Operasi</t>
+          <t>Milik Pelanggan</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
           <t>Boundary_External; source evidence</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
         </is>
       </c>
     </row>
@@ -5575,22 +6482,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BSH</t>
+          <t>DKSBI</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BSH (KTT / customer asset)</t>
+          <t>Durikosambi</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>CKDRU</t>
+          <t>KMBGN</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>KTT / customer</t>
+          <t>Boundary / external</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -5603,12 +6510,401 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Milik Pelanggan</t>
+          <t>Beroperasi</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
           <t>Boundary_External; source evidence</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PKTGN</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Petukangan</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>KMBGN</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Boundary / external</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Boundary_External; source evidence</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ABDGP</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Abadi Guna Papan</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>DNYSA</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Boundary / external</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Boundary_External; source evidence</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>MPANG</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Mampang</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>DNYSA</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Boundary / external</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Boundary_External; source evidence</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SVRNA</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Suvarna Sutra</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>CKUPA</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>SUTT</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PSKMS</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Pasar Kemis</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>CKUPA</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>SUTT</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>DKSBI</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Durikosambi</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>CNKNG</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>SUTT</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PKTGN</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Petukangan</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>SNYAN</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>SKTT</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Belum Operasi</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ABDGP</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Abadi Guna Papan</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>SNYAN</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>SKTT</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Belum Operasi</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>KEMBANGAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>JTAKE</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Jatake</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>CKUPA</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>SUTT</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Belum Operasi</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>BALARAJA</t>
         </is>
       </c>
     </row>

</xml_diff>